<commit_message>
2026 03 02 realise
</commit_message>
<xml_diff>
--- a/borchestra_abils.xlsx
+++ b/borchestra_abils.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C159"/>
+  <dimension ref="A1:C209"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,2118 +436,3653 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sloppy Haymaker</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr"/>
+          <t>Pike_A</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Pike</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Deal damage equal to this party member's Resonance + 3 to the Opposing enemy. Lose Resonance equal to the damage dealt.</t>
+          <t>Deal an Agonizing amount of Damage to the Left and Right party members not Opposing this enemy.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Amateur Haymaker</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
+          <t>Torrent_A</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Torrent</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Deal damage equal to this party member's Resonance + 4 to the Opposing enemy. Lose Resonance equal to the damage dealt.</t>
+          <t>Moves all Party members away from this enemy.
+Deals a Little amount of Indirect damage to the Opposing Party members.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Practiced Haymaker</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
+          <t>GoFish_A</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Go Fish</t>
+        </is>
+      </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Deal damage equal to this party member's Resonance + 6 to the Opposing enemy. Lose Resonance equal to the damage dealt.</t>
+          <t>Deal a Painful amount of Damage to a random Opposing party member, and destroy their held item.
+If successful produce a random \!fish\! on combat end.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Perfect Haymaker</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
+          <t>MimicSwipe_A</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Swipe</t>
+        </is>
+      </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Deal damage equal to this party member's Resonance + 7 to the Opposing enemy. Lose Resonance equal to the damage dealt.</t>
+          <t>Move this Enemy to the Left or Right.
+Deals a Painful amount of damage to the Opposing party member, if successful steals the Opposing party member's item.
+If you are out of items, Flees.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Flimsy Stonecutter</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
+          <t>MimicInk_A</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Ink</t>
+        </is>
+      </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>If the Left ally has no Shield, deal 4 damage to them and apply 8 Shield. If they have Shield, heal them for their Shield and remove it.</t>
+          <t>Inflicts 1-2 Oil-Slicked to the Opposing party member.
+Deals a Painful amount of damage to the Opposing party member.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Flimsy Stonecutter</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
+          <t>MimicSticky_A</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Sticky</t>
+        </is>
+      </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>If the Left ally has no Shield, deal 3 damage to them and apply 10 Shield. If they have Shield, heal them for their Shield and remove it.</t>
+          <t>Steals 1 coin from the Left and Right party members. Applies 1 Constricted to the Left and Right party members.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Flimsy Stonecutter</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
+          <t>MimicSnag_A</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Snag</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>If the Left ally has no Shield, deal 2 damage to them and apply 12 Shield. If they have Shield, heal them for their Shield and remove it.</t>
+          <t>Move this Enemy to the Left or Right.
+Deals a Painful amount of damage to the Opposing party member, if successful steal 5 coins. 
+If you are out of money, Flees.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Flimsy Stonecutter</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
+          <t>Reverberate_A</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Reverberate</t>
+        </is>
+      </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>If the Left ally has no Shield, deal 2 damage to them and apply 14 Shield. If they have Shield, heal them for their Shield and remove it.</t>
+          <t>Lowers the max healths of the Left and Right party members by 3 and applies 2 Ruptured to them.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Rumbling Tremors</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
+          <t>MimicSmackdown_A</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Smackdown</t>
+        </is>
+      </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Deal damage equal to this party member's Resonance + 1 to the Left and Right enemies. Lose all Resonance.</t>
+          <t>Deals a Painful amount damage to the Opposing party member. Steal the Opposing party member's item and moves to the Left or Right.
+If you are out of items, Flees.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Quaking Tremors</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
+          <t>MimicSouvenir_A</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Souvenir</t>
+        </is>
+      </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Deal damage equal to this party member's Resonance + 3 to the Left and Right enemies. Lose all Resonance.</t>
+          <t>Moves to the Left twice or to the Right twice. 50% chance to steal the Far Left and Far Right party members' items.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Shattering Tremors</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
+          <t>MimicShakedown_A</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Shakedown</t>
+        </is>
+      </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Deal damage equal to this party member's Resonance + 4 to the Left and Right enemies. Lose all Resonance.</t>
+          <t>Deals a Painful amount damage to the Opposing party member. Steals 3 coins from the Opposing party member and moves to the Left or Right.
+If you are out of money, Flees.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Splitting Tremors</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr"/>
+          <t>StreetPerformance_A</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Street Performance</t>
+        </is>
+      </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Deal damage equal to this party member's Resonance + 5 to the Left and Right enemies. Lose all Resonance.</t>
+          <t>Moves to the Left twice or to the Right twice. Steals 2 coins from the Far Left and Far Right party members.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Blindly Fumble</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
+          <t>ArtificialLycanthropy_A_0</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Artificial Lycanthropy</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Deal 8 damage to the Opposing enemy.
-If this kills, a random enemy takes the excess damage indirectly.</t>
+          <t>Perform 5 random enemy moves back to back.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Blindly Flail</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr"/>
+          <t>FuckThis_A_0</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>F@#% This!</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Deal 10 damage to the Opposing enemy.
-If this kills, a random enemy takes the excess damage indirectly.</t>
+          <t>Flee.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Blindly Tussle</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr"/>
+          <t>EnemyDiscipline_A</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Discipline</t>
+        </is>
+      </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Deal 12 damage to the Opposing enemy.
-If this kills, a random enemy takes the excess damage indirectly.</t>
+          <t>Deal an Agonizing amount of damage to the opposing party member. Damage will spread indirectly to the party members left and right.
+Deal a Painful amount of damage to the left and right enemy</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Blindly Rumble</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
+          <t>Whip_A</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Whip</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Deal 14 damage to the Opposing enemy.
-If this kills, a random enemy takes the excess damage indirectly.</t>
+          <t>Move this enemy left or right.
+Inflict 2 Frail to the opposing party member.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Unforgiving Splitter</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
+          <t>UnravelThem_A</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Unravel Them</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Deal 6 damage to the Opposing enemy.
-If this kills, deal 5 damage to the left and right enemies.</t>
+          <t>Deal a Painful amount of damage to the Left and Right party members.
+Deal Damage equal to how much damage the Left and Right party member took, to the Opposing party member.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ruthless Splitter</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
+          <t>RamtheRight_A</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Ram the Right</t>
+        </is>
+      </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Deal 7 damage to the Opposing enemy.
-If this kills, deal 8 damage to the left and right enemies.</t>
+          <t>Deals a Painful amount of damage to the Right Opposing party member.
+Apply 1 Infestation to the Left Opposing party member.
+Moves this enemy to the Right.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Cruel Splitter</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
+          <t>CrushtheLeft_A</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Crush the Left</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Deal 8 damage to the Opposing enemy.
-If this kills, deal 11 damage to the left and right enemies.</t>
+          <t>Deals a Painful amount of damage to the Left Opposing party member.
+Apply 1 Infestation to the Right Opposing party member.
+Moves this enemy to the Left.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Merciless Splitter</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
+          <t>Herbivore_A</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Herbivore</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Deal 9 damage to the Opposing enemy.
-If this kills, deal 14 damage to the left and right enemies.</t>
+          <t>Removes all Infestation from the Opposing party members and distributes it evenly among all other enemies.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Blemish the Pigment</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
+          <t>Headbutt_A</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Headbutt</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Deals damage to the Opposing enemy according to their health color.
-Grey or red health enemies recieve 6 damage, purple health enemies recieve 10 damage, and blue or yellow health enemies recieve 12 damage.</t>
+          <t>Deal a Painful amount of Damage to the Opposing party member.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Disfigure the Pigment</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr"/>
+          <t>ChapmanInfest_A</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Infest</t>
+        </is>
+      </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Deals damage to the Opposing enemy according to their health color.
-Grey-health enemies recieve 6 damage, red-health enemies recieve 8 damage, purple health enemies recieve 12 damage, and blue or yellow health enemies recieve 16 damage.</t>
+          <t>Apply 3 infestation spread randomly throughout every enemy.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Mangle the Pigment</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr"/>
+          <t>FruitsthatFeast_A</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Fruits that Feast</t>
+        </is>
+      </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Deals damage to the Opposing enemy according to their health color.
-Grey-health enemies recieve 6 damage, red-health enemies recieve 10 damage, purple health enemies recieve 15 damage, and blue or yellow health enemies recieve 20 damage.</t>
+          <t>Deals almost no damage to this enemy. Heals all other enemies an amount equal to the damage dealt.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Mutilate the Pigment</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr"/>
+          <t>FloodsFromTheGarden_A</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Floods from the Garden</t>
+        </is>
+      </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Deals damage to the Opposing enemy according to their health color.
-Grey-health enemies recieve 6 damage, red-health enemies recieve 12 damage, purple health enemies recieve 20 damage, and blue or yellow health enemies recieve 22 damage.</t>
+          <t>Apply 0-3 shield to every enemy position besides own.
+Consume 3 Purple pigment.
+If 3 pigment have been consumed, Curse the party member with the highest health. Ignores already Cursed party members.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Drink Under</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr"/>
+          <t>AbandonAllHope_A</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Abandon All Hope</t>
+        </is>
+      </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Deal 3 indirect damage to this party member. Deal 10 indirect damage to the Opposing enemy. Both spread.</t>
+          <t>Deal a Painful amount of damage to the Left and Right party members.
+Consume 3 Red pigment.
+If 3 pigment have been consumed, deal a Lethal amount of Damage to all party members and destroy this enemy.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Haphazardly Maul</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr"/>
+          <t>BowlsOfFire_A</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Bowls of Fire</t>
+        </is>
+      </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Deal 6 damage to the Opposing Enemy. If they are Constricted, inflict 2 Constricted to the Left and Right slots and then deal 3 damage to the Left and Right enemies.</t>
+          <t>Inflict 1 Fire to 1-2 Random party member positions.
+Consume 3 Yellow pigment.
+If 3 pigment have been consumed, inflict 1 Fire to all party member positions, and 1 Oil-slicked to 3 random party members.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Messily Maul</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr"/>
+          <t>RapturousRupture_A</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Rapturous Rupture</t>
+        </is>
+      </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Deal 8 damage to the Opposing Enemy. If they are Constricted, inflict 2 Constricted to the Left and Right slots and then deal 5 damage to the Left and Right enemies.</t>
+          <t>Move Left or Right and inflict 2 Ruptured to the Opposing party member.
+Consume 3 Blue pigment.
+If 3 pigment have been consumed, inflict 1 Ruptured to all party members.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Deliberately Maul</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr"/>
+          <t>Rattle_A_0</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Rattle</t>
+        </is>
+      </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Deal 9 damage to the Opposing Enemy. If they are Constricted, inflict 3 Constricted to the Left and Right slots and then deal 7 damage to the Left and Right enemies.</t>
+          <t>Deal 3 damage to the Opposing enemy 5 times.
+20% chance to deal 2 Indirect damage instead each time.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Methodically Maul</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr"/>
+          <t>KnightsFocus_A_0</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Knight's Focus</t>
+        </is>
+      </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Deal 10 damage to the Opposing Enemy. If they are Constricted, inflict 3 Constricted to the Left and Right slots and then deal 8 damage to the Left and Right enemies.</t>
+          <t>Gain Focus</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Prickly Hedgehog</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr"/>
+          <t>KnightLance_A_0</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Speedy Lance</t>
+        </is>
+      </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Deal 5 indirect damage to the Left and Right enemies, and 4 direct damage to the Opposing enemy. Inflict 1 Constricted to the Left and Right enemies.</t>
+          <t>Deal 6 damage to the Left and RIght enemy.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Spiky Hedgehog</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr"/>
+          <t>KnightLance_A_1</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Steadfast Lance</t>
+        </is>
+      </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Deal 6 indirect damage to the Left and Right enemies, and 5 direct damage to the Opposing enemy. Inflict 2 Constricted to the Left and Right enemies.</t>
+          <t>Deal 8 damage to the Left and RIght enemy.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Piercing Hedgehog</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr"/>
+          <t>KnightLance_A_2</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Brave Lance</t>
+        </is>
+      </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Deal 7 indirect damage to the Left and Right enemies, and 6 direct damage to the Opposing enemy. Inflict 2 Constricted to the Left and Right enemies.</t>
+          <t>Deal 10 damage to the Left and RIght enemy.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Penetrating Hedgehog</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr"/>
+          <t>KnightLance_A_3</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Holy Lance</t>
+        </is>
+      </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Deal 9 indirect damage to the Left and Right enemies, and 8 direct damage to the Opposing enemy. Inflict 3 Constricted to the Left and Right enemies.</t>
+          <t>Deal 12 damage to the Left and RIght enemy.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Weak Intent</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr"/>
+          <t>KnightsChivalry_A_0</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Fading Chivalry</t>
+        </is>
+      </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Inflict 2 Constricted and 1 Frail to the Opposing enemy.</t>
+          <t>Apply 5 Shield to the lowest health party member(s).</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Middling Intent</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr"/>
+          <t>KnightsChivalry_A_1</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Squire's Chivalry</t>
+        </is>
+      </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Inflict 2 Constricted and 1 Frail to the Opposing and Left enemies.</t>
+          <t>Apply 7 Shield to the lowest health party member(s).</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Decisive Intent</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr"/>
+          <t>KnightsChivalry_A_2</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Warrior's Chivalry</t>
+        </is>
+      </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Inflict 2 Constricted and 1 Frail to the Opposing, Left, and Right enemies.</t>
+          <t>Apply 9 Shield to the lowest health party member(s).</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Killer Intent</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr"/>
+          <t>KnightsChivalry_A_3</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Hero's Chivalry</t>
+        </is>
+      </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Inflict 3 Constricted and 1 Frail to the Opposing, Left, and Right enemies.</t>
+          <t>Apply 10 Shield to the lowest health party member(s).</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Pummel their Armor</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr"/>
+          <t>CopperCough_A</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Copper Cough</t>
+        </is>
+      </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Deal 6 damage to the Opposing enemy. Deal double if this party member is in the center position.
-Move the Opposing enemy towards the center of the field.</t>
+          <t>Produce 1 Coin and Die unceremoniously.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Pummel their Guard</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr"/>
+          <t>SquidSlap_A</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Squid Slap</t>
+        </is>
+      </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Deal 8 damage to the Opposing enemy. Deal double if this party member is in the center position.
-Move the Opposing enemy towards the center of the field.</t>
+          <t>Deals a Painful amount of damage to the Opposing party member.
+Moves the Opposing party member to the Left or Right.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Pummel their Weakspot</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr"/>
+          <t>Mishandle_A</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Mishandle</t>
+        </is>
+      </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Deal 10 damage to the Opposing enemy. Deal double if this party member is in the center position.
-Move the Opposing enemy towards the center of the field.</t>
+          <t>Deals a Little amount of damage to the Opposing party member.
+Inflict 2 Ruptured to the Opposing party member.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Pummel their Achilles</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr"/>
+          <t>SlipperyStruggle_A</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Slippery Struggle</t>
+        </is>
+      </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Deal 12 damage to the Opposing enemy. Deal double if this party member is in the center position.
-Move the Opposing enemy towards the center of the field.</t>
+          <t>Deals a Painful damage to a random party member Opposing or to the Left or Right of this enemy.
+Inflict 3 Oil-Slicked to the Opposing party Member.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Menacingly Intimidate</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr"/>
+          <t>BirdOfPrey_A</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Bird of Prey</t>
+        </is>
+      </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Deal 4 damage to the Opposing enemy and inflict 1 Scar. If this party member is on the edge of the field, deal double damage and inflict another Scar. 
-Move the Opposing enemy towards the center of the field.</t>
+          <t>Deals a Painful amount of damage to the highest health party member(s). Applies 2 Frail to the highest health party member(s).</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Terrifying Intimidate</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr"/>
+          <t>Together_A</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Together</t>
+        </is>
+      </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Deal 5 damage to the Opposing enemy and inflict 1 Scar. If this party member is on the edge of the field, deal double damage and inflict another 2 Scars. 
-Move the Opposing enemy towards the center of the field.</t>
+          <t>Inflict 2 Linked to the Opposing party member and 2 Linked to this enemy.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Paralyzing Intimidate</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr"/>
+          <t>Pressure_A</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Pressure</t>
+        </is>
+      </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Deal 6 damage to the Opposing enemy and inflict 1 Scar. If this party member is on the edge of the field, deal double damage and inflict another 2 Scars. 
-Move the Opposing enemy towards the center of the field.</t>
+          <t>Increases the duration of all negative status effects inflicted to All party members by 2.
+Decreases the Opposing party member's maximum health by 4.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Heart-Stopping Intimidate</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr"/>
+          <t>Headache_A</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Headache</t>
+        </is>
+      </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Deal 6 damage to the Opposing enemy and inflict 1 Scar. If this party member is on the edge of the field, deal double damage and inflict another 3 Scars. 
-Move the Opposing enemy towards the center of the field.</t>
+          <t>Applies 2 Ruptured to the Far Left and Far Right party members. Deals barely any damage to the Far Left and Far Right party members.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Unwieldy Buckler</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr"/>
+          <t>Wave_A</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Wave</t>
+        </is>
+      </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Deal 3 damage to the enemy Opposing the lowest health party member(s), then apply 6 Shield to that party member's position.</t>
+          <t>Spawn 2 Tentacles.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Basic Buckler</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr"/>
+          <t>SquidCry_A</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Cry</t>
+        </is>
+      </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Deal 4 damage to the enemy Opposing the lowest health party member(s), then apply 8 Shield to that party member's position.</t>
+          <t>This enemy cries and produces 1 Blue Pigment. Applies 2 Oil Slicked to the Opposing party member.
+\!It ain't easy being greasy.\!</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Formidable Buckler</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr"/>
+          <t>SquareUp_A</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Square Up</t>
+        </is>
+      </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Deal 5 damage to the enemy Opposing the lowest health party member(s), then apply 10 Shield to that party member's position.</t>
+          <t>Retracts all current tentacles and summons new ones equal to the amount retracted.
+If there are no Tentacles present produce 1 Blue Pigment.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Impregnable Buckler</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr"/>
+          <t>Violator_A</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Violator</t>
+        </is>
+      </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Deal 6 damage to the enemy Opposing the lowest health party member(s), then apply 12 Shield to that party member's position.</t>
+          <t>Deals a Painful amount of damage to the Opposing party member.
+Spawn as many Deer as possible.
+If spawning was successful lower the Doula's damage by 1, and lower its Multi-Attack by 1 as well.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Eerie Smoothing</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr"/>
+          <t>NoBruises_A</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>DoulaMultiAttack</t>
+        </is>
+      </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Heal the Left and Right allies 2 health.</t>
+          <t>Increase the Doula's Attack damage by 2.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Specter's Smoothing</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr"/>
+          <t>NoWords_A</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>No Words</t>
+        </is>
+      </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Heal the Left and Right allies 3 health.</t>
+          <t>Increase the Doula's MultiAttack by 1.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Phantasm's Smoothing</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr"/>
+          <t>Gestate_A</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Gestate</t>
+        </is>
+      </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Heal the Left, Far Left, Right, and Far Right allies 4 health.</t>
+          <t>Apply 3 Scars to every deer.
+\!It shouldn't have been you\!</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Poltergeist's Smoothing</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr"/>
+          <t>Regret_A</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>DoulaAttack</t>
+        </is>
+      </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Heal the Left, Far Left, Right, and Far Right allies 5 health.</t>
+          <t>Instantly kill the Opposing party member.
+If succesful reset all of Doula's values.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Poke The Skin</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr"/>
+          <t>IntrudingOsteophagy_A</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Intruding Osteophagy</t>
+        </is>
+      </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Deal 2 damage and inflict 2 Ruptured to the Opposing enemy. Move the Opposing enemy to the Left or Right.</t>
+          <t>Deal a Painful amount of Damage to the Opposing enemy.
+Inflict 2 Ruptured to the Opposing enemy.
+Decrease Doula's damage by 1, 50% chance to decrease Doula's MultiAttack by 1 as well.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Poke The Arteries</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr"/>
+          <t>IntheHeadlights_A</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>In the Headlights</t>
+        </is>
+      </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Deal 3 damage and inflict 3 Ruptured to the Opposing enemy. Move the Opposing enemy to the Left or Right.</t>
+          <t>This enemy forfeits it's turn.
+\!Got caught\!</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Poke The Muscles</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr"/>
+          <t>MeleeSwing_A_0</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Melee Swing</t>
+        </is>
+      </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Deal 4 damage and inflict 4 Ruptured to the Opposing enemy. Move the Opposing enemy to the Left or Right.</t>
+          <t>Deal 5 Damage to the Opposing enemy.
+Small chance to Randomly crit and deal 20 Damage instead.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Poke The Nerves</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr"/>
+          <t>Ascension_A_0</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Ascension</t>
+        </is>
+      </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Deal 5 damage and inflict 5 Ruptured to the Opposing enemy. Move the Opposing enemy to the Left or Right.</t>
+          <t>This party member enters the opposing enemy. Adds an amount of Parasitism equal to this party member's current health to the Opposing enemy.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Flimsy Vindication</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr"/>
+          <t>SameRoutine_A_0</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Same Routine</t>
+        </is>
+      </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Remove 1 Constricted from this party member's position and restore their movement. 
-Apply 3 Shield to this party member's position.</t>
+          <t>Cancel one of the Opposing enemy's moves.
+Stun this party member.
+20% chance to stun another random party member as well.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Shoddy Vindication</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr"/>
+          <t>RecordScratch_A_0</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Record Scratch</t>
+        </is>
+      </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Remove 1 Constricted from this party member's position and restore their movement. 
-Apply 5 Shield to this party member's position.</t>
+          <t>Cancel one of the Opposing enemy's moves.
+50% chance to Refresh this party member.
+20% chance to scratch the record.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Half-Baked Vindication</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr"/>
+          <t>LenghtyExcommunication_A_0</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Lenghty Excommunication</t>
+        </is>
+      </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Remove 1 Constricted from this party member's position and restore their movement. 
-Apply 7 Shield to this party member's position.</t>
+          <t>Increases the opposing enemy's \!Exorcism\! counter by 1.
+Once the counter reaches how much maximum health the enemy has divided by 10, instantly kill it.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Reasonable Vindication</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr"/>
+          <t>GorillaSprint_A</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Gorilla Sprint</t>
+        </is>
+      </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Remove 1 Constricted from this party member's position and restore their movement. 
-Apply 9 Shield to this party member's position.</t>
+          <t>Move to the Left or Right as far as possible.
+Deal an Agonizing amount damage to the Opposing party member.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Decay the Flesh</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr"/>
+          <t>Mortify_A</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Mortify</t>
+        </is>
+      </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Deal 5 damage to the Left and Right enemies. If this kills either enemy, this party member is indirectly healed by the amount of Tumors they have plus 1. Costs 1 Tumor to use.</t>
+          <t>Inflict 2 Constricted to the Farthest enemy(s) positions.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Decay the Bone</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr"/>
+          <t>FallApart_A_0</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Fall Apart</t>
+        </is>
+      </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Deal 7 damage to the Left and Right enemies. If this kills either enemy, this party member is indirectly healed by the amount of Tumors they have plus 1. Costs 1 Tumor to use.</t>
+          <t>Inflict 1 Scar to this party member.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Decay the Innards</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr"/>
+          <t>GhastlyCryPA_A</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Ghastly Cry</t>
+        </is>
+      </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Deal 8 damage to the Left and Right enemies. If this kills either enemy, this party member is indirectly healed by the amount of Tumors they have plus 2. Costs 1 Tumor to use.</t>
+          <t>Retribution for violence against the host.
+Deals a Little amount of damage to the Opposing party member. 
+Applies 2 Ruptured and 2 Oil Slicked to the Opposing party member.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Decay the Life</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr"/>
+          <t>Flick_A</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Flick</t>
+        </is>
+      </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Deal 10 damage to the Left and Right enemies. If this kills either enemy, this party member is indirectly healed by the amount of Tumors they have plus 2. Costs 1 Tumor to use.</t>
+          <t>Deals a Little amount of indirect damage to the Opposing party member. Set the Opposing party member's max health to equal their current health.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Mould the Form</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr"/>
+          <t>EctoplasmicEmesis_A</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Ectoplasmic Emesis</t>
+        </is>
+      </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Indirectly heal this party member for the amount of Tumors they have. 
-Apply 6 Shield to this party member if they have 2+ Tumors. Apply Focused to this party member if they have 3+ Tumors. 
-Remove all Tumors.</t>
+          <t>This enemy produces one Purple, and one Blue pigment.
+\!Point of study among experts nowhere\!</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Mould the Body</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr"/>
+          <t>GhastlyCry_A</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Ghastly Cry</t>
+        </is>
+      </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Indirectly heal this party member for the amount of Tumors they have. 
-Apply 8 Shield to this party member if they have 2+ Tumors. Apply Focused to this party member if they have 3+ Tumors. 
-Remove all Tumors.</t>
+          <t>Attempt to summon an Unflarb.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Mould the Soul</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr"/>
+          <t>AllureofEternity_A</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Allure of Eternity</t>
+        </is>
+      </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Indirectly heal this party member for the amount of Tumors they have times two. 
-Apply 12 Shield to this party member if they have 2+ Tumors. Apply Focused to this party member if they have 3+ Tumors. 
-Remove all Tumors.</t>
+          <t>Attract an Enemy for assistance. If there are no Enemies attract 2 Instead.
+\!Too good to be true...\!</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Mould into Perfection</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr"/>
+          <t>OnewiththeDivine_A</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>One with the Divine</t>
+        </is>
+      </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Indirectly heal this party member for the amount of Tumors they have times two. 
-Apply 15 Shield to this party member if they have 2+ Tumors. Apply Focused to this party member if they have 3+ Tumors. 
-Remove all Tumors.</t>
+          <t>Apply 3 Divine protection to the Left and Right enemies.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Fracture into Pieces</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr"/>
+          <t>PrismaticParasite_A</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Prismatic Parasite</t>
+        </is>
+      </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Deal 6 damage to the Opposing enemy, dealing double damage if they have Frail. Afterwards, inflict 1 Frail on the Opposing enemy. 
-Costs 2 Tumors.</t>
+          <t>Consume 1 Pigment of each colour.
+\!The little that's left...\!</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Shatter into Wreckage</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr"/>
+          <t>MudFever_A</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Mud Fever</t>
+        </is>
+      </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Deal 8 damage to the Opposing enemy, dealing double damage if they have Frail. Afterwards, inflict 2 Frail on the Opposing enemy. 
-Costs 2 Tumors.</t>
+          <t>Grant the far Left and the Far right enemy a Bonus action.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Sunder into Fragments</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr"/>
+          <t>Salvation_A</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Salvation</t>
+        </is>
+      </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Deal 10 damage to the Opposing enemy, dealing double damage if they have Frail. Afterwards, inflict 2 Frail on the Opposing enemy. 
-Costs 2 Tumors.</t>
+          <t>Fully heal the Left and Right enemy.
+Inflict 2 Frail to the Left and Right enemy.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Split into Molecules</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr"/>
+          <t>Flay_A</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Flay</t>
+        </is>
+      </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Deal 12 damage to the Opposing enemy, dealing double damage if they have Frail. Afterwards, inflict 3 Frail on the Opposing enemy. 
-Costs 2 Tumors.</t>
+          <t>Deal an Agonizing amount of damage to the enemy(s) with the lowest health. If an enemy is killed, become cozy.</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>Condemn to Pain</t>
-        </is>
-      </c>
+      <c r="A75" t="inlineStr"/>
       <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr">
         <is>
-          <t>If the Opposing enemy is the target of this party member's Gaze, deal 10 damage to them. 
-Otherwise, deal 3-5 damage to them.</t>
+          <t>Upon death this enemy has a 60% chance of being stripped naked.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Condemn to Suffering</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr"/>
+          <t>Lunge_A</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Lunge</t>
+        </is>
+      </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>If the Opposing enemy is the target of this party member's Gaze, deal 12 damage to them. 
-Otherwise, deal 3-7 damage to them.</t>
+          <t>This enemy moves to the Left or Right.
+Deal an Agonizing amount of damage to the Opposing party member.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Condemn to Torment</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr"/>
+          <t>StomachAcids_A</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Stomach Acids</t>
+        </is>
+      </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>If the Opposing enemy is the target of this party member's Gaze, deal 13 damage to them. 
-Otherwise, deal 5-9 damage to them.</t>
+          <t>Remove all shield from the Opposing position.
+Deal a Painful amount of damage to the Opposing party member.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Condemn to Oblivion</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr"/>
+          <t>Goblin13_A</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>hehehehehe</t>
+        </is>
+      </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>If the Opposing enemy is the target of this party member's Gaze, deal 15 damage to them. 
-Otherwise, deal 5-11 damage to them.</t>
+          <t>Chump</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Stoke Embers</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr"/>
+          <t>Goblin12_A</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>GET OUTTA HERE</t>
+        </is>
+      </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Inflict 1 Fire on the Left and Right slots, then deal 5 damage to them. If either target is Gazed, inflict Hellfire instead.</t>
+          <t>DUMB F*&amp;^</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Kindle Flames</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr"/>
+          <t>Goblin11_A</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>HAHA</t>
+        </is>
+      </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Inflict 1 Fire on the Left and Right slots, then deal 8 damage to them. If either target is Gazed, inflict Hellfire instead.</t>
+          <t>TAKE THAT YOU JERK</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Spark Fires</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr"/>
+          <t>Goblin10_A</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>alright ready?</t>
+        </is>
+      </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Inflict 1 Fire on the Left and Right slots, then deal 10 damage to them. If either target is Gazed, inflict Hellfire instead.</t>
+          <t>Here goes…</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Light Inferno</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr"/>
+          <t>Goblin13Alt_A</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>GET OUT</t>
+        </is>
+      </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Inflict 1-2 Fire on the Left and Right slots, then deal 11 damage to them. If either target is Gazed, inflict Hellfire instead.</t>
+          <t>OUT</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Hurtful Exposure</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr"/>
+          <t>Goblin11Alt_A</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Yeah alright there you go</t>
+        </is>
+      </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Deal 6 damage to the Opposing enemy and all enemies subject to this party member's Gaze. 
-Will not attack the Opposing enemy twice.</t>
+          <t>Now GET OUT</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Painful Exposure</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr"/>
+          <t>Goblin10Alt_A</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>alright ready?</t>
+        </is>
+      </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Deal 8 damage to the Opposing enemy and all enemies subject to this party member's Gaze. 
-Will not attack the Opposing enemy twice.</t>
+          <t>Here goes…</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Agonizing Exposure</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr"/>
+          <t>Goblin9_A</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Come here</t>
+        </is>
+      </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Deal 10 damage to the Opposing enemy and all enemies subject to this party member's Gaze. 
-Will not attack the Opposing enemy twice.</t>
+          <t>Stand in front of me and let me do my magic</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Torturous Exposure</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr"/>
+          <t>Goblin8_A</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>I was skeptical at first</t>
+        </is>
+      </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Deal 12 damage to the Opposing enemy and all enemies subject to this party member's Gaze. 
-Will not attack the Opposing enemy twice.</t>
+          <t>But you seem fine enough unlike other jerks that disturb me</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>QUICKLY GORGE</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr"/>
+          <t>Goblin7_A</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>yeah thats right</t>
+        </is>
+      </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Deal 10 damage to the Opposing enemy.
-If this kills, refresh this party member's movement and abilities.</t>
+          <t>I'm a MAGICAL goblin</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>INTENSELY GORGE</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr"/>
+          <t>Goblin6_A</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>sigh</t>
+        </is>
+      </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Deal 12 damage to the Opposing enemy.
-If this kills, refresh this party member's movement and abilities.</t>
+          <t>Alright sorry I got a bit aggressive there</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CRAZILY GORGE</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr"/>
+          <t>Goblin5_A</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Deal 16 damage to the Opposing enemy.
-If this kills, refresh this party member's movement and abilities.</t>
+          <t>...</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>THE GORGE</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr"/>
+          <t>Goblin4_A</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>never seen a goblin beat someone up?</t>
+        </is>
+      </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Deal 18 damage to the Opposing enemy.
-If this kills, refresh this party member's movement and abilities.</t>
+          <t>Well I'm gonna SHOW YOU</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>GOOFILY SLEEP</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr"/>
+          <t>Goblin3_A</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>how about I trample YOUR FACE</t>
+        </is>
+      </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Applies 4 Shield to this party member, then heals them 2 health.
-Gain a stack of Omega-Rested.</t>
+          <t>HUH? how's THAT sound?</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>LIGHTLY SLEEP</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr"/>
+          <t>Goblin2_A</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>come to MY trampling grounds</t>
+        </is>
+      </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Applies 6 Shield to this party member, then heals them 2 health.
-Gain a stack of Omega-Rested.</t>
+          <t>And give me that stupid look?</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>DEEP SLEEP</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr"/>
+          <t>Goblin1_A</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>What are you looking at?</t>
+        </is>
+      </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Applies 8 Shield to this party member, then heals them 2 health.
-Gain a stack of Omega-Rested.</t>
+          <t>Think you can just stroll up here?</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>THE SLEEP</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr"/>
+          <t>Plaster_A</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Plaster</t>
+        </is>
+      </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Applies 10 Shield to this party member, then heals them 2 health.
-Gain a stack of Omega-Rested.</t>
+          <t>Deal a Painful amount of Damage to the Left, Opposing, and Right party members.
+If this enemy has less than 50% health, deal that damage to only Opposing instead.
+Produce 1 Pigment of the Opposing party member's Health color.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>PATCH-UP ESSENCE</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr"/>
+          <t>Cling_A</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Cling</t>
+        </is>
+      </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Heal the Left party member 4 health.
-If this brings them to full health, refresh this party member's movement and abilities.</t>
+          <t>Produce 3 Pigment of the Opposing party member's Health color.
+If there is no Opposing party member deal a Painful amount of damage to this enemy.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>REJUVENATING ESSENCE</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr"/>
+          <t>IdentityCrisis_A</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Identity Crisis</t>
+        </is>
+      </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Heal the Left party member 6 health.
-If this brings them to full health, refresh this party member's movement and abilities.</t>
+          <t>33% chance to apply Cursed, 5 Oil-Slicked, 2 Fire, or 3 Ruptured each to the Opposing party member.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>MENDING ESSENCE</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr"/>
+          <t>Clamp_A</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Clamp</t>
+        </is>
+      </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Heal the Left party member 8 health.
-If this brings them to full health, refresh this party member's movement and abilities.</t>
+          <t>Deals a Painful Amount of damage to the Left and Right party members. If this enemy has less than 50% health, deals an Agonizing amount instead. 
+This enemy consumes 2 pigment not of this enemy's health color.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>THE ESSENCE</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr"/>
+          <t>Slurm_A</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Slurm</t>
+        </is>
+      </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Heal the Left party member 10 health.
-If this brings them to full health, refresh this party member's movement and abilities.</t>
+          <t>This enemy consumes 3 Pigment not of this enemy's health color. Deals a little amount of damage to this enemy for each pigment consumed.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Paltry Medicate</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr"/>
+          <t>FacelessCrowd_A</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Faceless Crowd</t>
+        </is>
+      </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Remove all Status Effects and Field Effects from the Left and Right Allies, then heal them 5 health.</t>
+          <t>Applies 1 Fire and 2 Ruptured to the Left and Right party member positions, deals a Painful amount of damage to them, and applies 4 Shield to the Left and Right enemy positions.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Novice Treatment</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr"/>
+          <t>ChaosDance_A</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Chaos Dance</t>
+        </is>
+      </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Remove all Status Effects and Field Effects from the Left and Right Allies, then heal them 6 health.</t>
+          <t>\!*clap, clap!*\!
+50% chance to inflict 1 Ruptured to each party member, and then shuffle all party members.
+Inflict 1 Scar and 1 Ruptured to all other enemies.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Learned Cure</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr"/>
+          <t>ViolentManipulation_A</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Violent Manipulation</t>
+        </is>
+      </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Remove all Status Effects and Field Effects from the Left and Right Allies, then heal them 8 health.</t>
+          <t>\!Stand your GROOOOUND WHILE FIGHTING ME!\!
+Deal a Painful amount of damage to the Left and Right party member, and a Painful amount of damage to the Left and Right enemy.
+Apply 10 Shield to this enemy's position.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Expert Cleanse</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr"/>
+          <t>ViolentAlteration_A</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Violent Alteration</t>
+        </is>
+      </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Remove all Status Effects and Field Effects from the Left and Right Allies, then heal them 9 health.</t>
+          <t>\!Am I being USURPED BY P#!$*ES!?\!
+Deal a Painful amount of damage to the Far Left and Far Right party member and a Painful amount of damage to the Far Left and Far Right enemy.
+Apply 10 Shield to this enemy's position.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Partial Nullify</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr"/>
+          <t>DaggerTongue_A</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Dagger Tongue</t>
+        </is>
+      </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Reroll one of the Opposing enemy's abilities. 5% chance per enemy to remove one of the Opposing enemy's abilities.</t>
+          <t>\!Impression and hatred are FAR from synonyms, you goddamn-\!
+Deal an Agonizing amount of damage to the Opposing party member, Move all other enemies to the Left or Right.
+Apply 7 shield to this enemy's position.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Impressive Nullify</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr"/>
+          <t>PlayAlong_A</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Play Along</t>
+        </is>
+      </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Reroll one of the Opposing enemy's abilities. 7% chance chance per enemy to remove one of the Opposing enemy's abilities.</t>
+          <t>\!I do not use buzzwords, trust-you-me.\!
+This enemy performs a random one of its abilities.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Grand Nullify</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr"/>
+          <t>SmugSuperiority_A</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Smug Superiority</t>
+        </is>
+      </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Reroll two of the Opposing enemy's abilities. 9% chance chance per enemy to remove two of the Opposing enemy's abilities.</t>
+          <t>Make Intijar perform an additional move. 
+\!These illogical actions of yours...well, I find them amusing\!.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Magnificent Nullify</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr"/>
+          <t>DivineImitation_A</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Imitation</t>
+        </is>
+      </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Reroll two of the Opposing enemy's abilities. 12% chance chance per enemy to remove two of the Opposing enemy's abilities.</t>
+          <t>Apply Focus and 2 Divine Protection to Intijar.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Cruel Affliction</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr"/>
+          <t>Jag_A</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Jag</t>
+        </is>
+      </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Inflict Cursed and 1 Frail to the Opposing enemy.</t>
+          <t>Inflict 2 Rupture to the Left and Right party members.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Baleful Affliction</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr"/>
+          <t>Spill_A</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Spill</t>
+        </is>
+      </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Inflict Cursed, 1 Frail, and 1 Scar to the Opposing enemy.</t>
+          <t>Produces 1 Pigment of this enemy's health colour.
+Deals a Little amount of damage to this enemy.</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>Malicious Affliction</t>
-        </is>
-      </c>
-      <c r="B109" t="inlineStr"/>
+      <c r="A109" t="inlineStr"/>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Reactive</t>
+        </is>
+      </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Inflict Cursed, 1 Frail, 1 Scar, and 2 Ruptured to the Opposing enemy.</t>
+          <t>Upon receiving Damage, this enemy will summon an enemy in retaliation.</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Malicious Affliction</t>
-        </is>
-      </c>
-      <c r="B110" t="inlineStr"/>
+          <t>Castigate_A</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Castigate</t>
+        </is>
+      </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Inflict Cursed, 1 Frail, 2 Scars, and 3 Ruptured to the Opposing enemy.</t>
+          <t>Deals a Painful amount of damage to the Opposing party member.
+Damage spreads indirectly to the Party members on the Left or Right.</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Quickly Gorge</t>
-        </is>
-      </c>
-      <c r="B111" t="inlineStr"/>
+          <t>Centralize_A</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Centralize</t>
+        </is>
+      </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Deal 5 damage to the Opposing enemy.
-If this kills, refresh this party member.</t>
+          <t>Summon a random rock.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Intensely Gorge</t>
-        </is>
-      </c>
-      <c r="B112" t="inlineStr"/>
+          <t>Brainstorm_A</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Brainstorm</t>
+        </is>
+      </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Deal 6 damage to the Opposing enemy.
-If this kills, refresh this party member.</t>
+          <t>Destroy every current Inanimate enemy.
+Deals damage equivalent to how much health the enemies had, the damage spreads equally among every party member.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Madly Gorge</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr"/>
+          <t>Maneuver_A</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Maneuver</t>
+        </is>
+      </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Deal 8 damage to the Opposing enemy.
-If this kills, refresh this party member.</t>
+          <t>Apply 2 Shields to the Left and Right Enemy position.
+Move this enemy to the Left or Right.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Unsatiably Gorge</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr"/>
+          <t>LeftMandible_A</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Left Mandible</t>
+        </is>
+      </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Deal 9 damage to the Opposing enemy.
-If this kills, refresh this party member.</t>
+          <t>Deals a Little amount of damage to the Far Left Opposing party member.
+Deals Barely any damage to the Left Opposing party member, and move that party member to the Right.
+Consume 1 pigment.</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Restless Sleep</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr"/>
+          <t>RightMandible_A</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Right Mandible</t>
+        </is>
+      </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Applies 2 Shield to this party member, then heals them 1 health.
-Gain a stack of Well-Rested.</t>
+          <t>Deals a Little amount of damage to the Far Right Opposing party member.
+Deals Barely any damage to the Right Opposing party member, and move that party member to the Left.
+Consume 1 pigment.</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Lightly Sleep</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr"/>
+          <t>MiddleMouthparts_A</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Middle Mouthparts</t>
+        </is>
+      </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Applies 3 Shield to this party member, then heals them 1 health.
-Gain a stack of Well-Rested.</t>
+          <t>Deals a little amount of damage to the Middlemost Opposing party member, move that party member to the Left or Right.
+\!Weirdly?\!</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Deeply Sleep</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr"/>
+          <t>Hurk_A</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Hurk</t>
+        </is>
+      </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Applies 4 Shield to this party member, then heals them 1 health.
-Gain a stack of Well-Rested.</t>
+          <t>Spawn a Festering Pile on the party member side. If unsuccessful, cure all Status effects on this enemy.</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Motionless Sleep</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr"/>
+          <t>FreshShed_A</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Fresh Shed</t>
+        </is>
+      </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Applies 5 Shield to this party member, then heals them 1 health.
-Gain a stack of Well-Rested.</t>
+          <t>Applies 0-2 Shield to All positions.
+Consume 2 pigment.
+Remove all Fire from Self positions.</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Essence Of Enduring</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr"/>
+          <t>ConductorFeelTheRhythmItem_A</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Feel the Rhythm</t>
+        </is>
+      </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Deal 5 damage to the Left and Opposing enemy. If less than 5 total damage is dealt, refresh this party member.</t>
+          <t>\!Becomes the instrument of the Ungod.\!</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Essence Of Vigor</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr"/>
+          <t>TongueBite_A</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Tongue Bite</t>
+        </is>
+      </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Deal 7 damage to the Left and Opposing enemy. If less than 7 total damage is dealt, refresh this party member.</t>
+          <t>Apply 3 Parasitism to the opposing party member.</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Essence Of Tenacity</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr"/>
+          <t>VoiceCrack_A</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Voice Crack</t>
+        </is>
+      </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Deal 9 damage to the Left and Opposing enemy. If less than 9 total damage is dealt, refresh this party member.</t>
+          <t>\!Ungoddamnit.
+Inflict 1 Scars to this enemy.</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Essence Of Spite</t>
-        </is>
-      </c>
-      <c r="B122" t="inlineStr"/>
+          <t>Reverence_A</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Reverence</t>
+        </is>
+      </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Deal 11 damage to the Left and Opposing enemy. If less than 11 total damage is dealt, refresh this party member.</t>
+          <t>Deal a Painful amount of Damage to the Opposing party members.</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Nostalgia</t>
-        </is>
-      </c>
-      <c r="B123" t="inlineStr"/>
+          <t>Travesty_A</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Travesty</t>
+        </is>
+      </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>This party member performs a random ability from another ally.</t>
+          <t>Inflict 1 Ruptured to All party members not opposing this enemy.</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Rough Chop</t>
-        </is>
-      </c>
-      <c r="B124" t="inlineStr"/>
+          <t>Vocal Tear_A</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Vocal Tear</t>
+        </is>
+      </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Deal 6-10 damage to the Opposing enemy. If no wrong pigment was used, heal this party member 4 health.</t>
+          <t>Inflict 1 Scar to this enemy. Deals damage to the Central Opposing party member equal to twice the amount of Scars this enemy has.</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Violent Chop</t>
-        </is>
-      </c>
-      <c r="B125" t="inlineStr"/>
+          <t>CountlessEyes_A</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Countless Eyes</t>
+        </is>
+      </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Deal 8-12 damage to the Opposing enemy. If no wrong pigment was used, heal this party member 5 health.</t>
+          <t>Move all party members away from this enemy.
+Apply 3 Fleeting to the Opposing party members, if they already have Fleeting increase it by 3.
+Move this enemy Left or Right twice.</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Maiming Chop</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr"/>
+          <t>CountlessTongues_A</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Countless Tongues</t>
+        </is>
+      </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Deal 10-14 damage to the Opposing enemy. If no wrong pigment was used, heal this party member 5 health.</t>
+          <t>Apply 2 Fleeting to the Opposing party members.
+If an Opposing party member already has Fleeting, Decrease their Fleeting by 1 instead.</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Neck-Breaking Chop</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr"/>
+          <t>Slobber_A</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Slobber</t>
+        </is>
+      </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Deal 12-16 damage to the Opposing enemy. If no wrong pigment was used, heal this party member 7 health.</t>
+          <t>Decreases the maximum health of the Opposing party members by 4.</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Forge Skin</t>
-        </is>
-      </c>
-      <c r="B128" t="inlineStr"/>
+          <t>EvenSludge_A</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Even Sludge</t>
+        </is>
+      </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Apply 4 Shield to self. If wrong pigment was used, this party member's non-slap abilities deal 1 extra damage.</t>
+          <t>Deals a Deadly amount of damage evenly spread between all positions not Opposing a Neoplasm.</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Forge Bone</t>
-        </is>
-      </c>
-      <c r="B129" t="inlineStr"/>
+          <t>TrudgeSlop_A</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Trudge Slop</t>
+        </is>
+      </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Apply 6 Shield to self. If wrong pigment was used, this party member's non-slap abilities deal 1 extra damage.</t>
+          <t>Moves this enemy to the Left if their health color is Yellow, or Right if their Health color is Red. Produce 1 Pigment of this enemy's health color.</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Forge Body</t>
-        </is>
-      </c>
-      <c r="B130" t="inlineStr"/>
+          <t>NauseatingChurn_A</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Nauseating Churn</t>
+        </is>
+      </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Apply 8 Shield to self. If wrong pigment was used, this party member's non-slap abilities deal 1 extra damage.</t>
+          <t>Slightly heal the nearest Left or Right enemy.</t>
         </is>
       </c>
     </row>
     <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>Forge Soul</t>
-        </is>
-      </c>
+      <c r="A131" t="inlineStr"/>
       <c r="B131" t="inlineStr"/>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Apply 11 Shield to self. If wrong pigment was used, this party member's non-slap abilities deal 1 extra damage.</t>
+          <t>Upon death this enemy spawns 2 Neoplasms.</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Cleave the Meat</t>
-        </is>
-      </c>
-      <c r="B132" t="inlineStr"/>
+          <t>SnappingGurgle_A</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Snapping Gurgle</t>
+        </is>
+      </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Deal 5 damage to the Left and Right enemies. If wrong pigment was used, instead deal 7 damage.</t>
+          <t>Produce 3-4 Pigment of this enemy's health colour.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Cleave the Flesh</t>
-        </is>
-      </c>
-      <c r="B133" t="inlineStr"/>
+          <t>MusicalBoil_A</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Musical Boil</t>
+        </is>
+      </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Deal 7 damage to the Left and Right enemies. If wrong pigment was used, instead deal 9 damage.</t>
+          <t>If this enemy's health color is Red, applies 2 Ruptured to all Opposing party members. If this enemy's health color is Yellow, applies 1 Fire to all Opposing party members.</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Cleave the Guts</t>
-        </is>
-      </c>
-      <c r="B134" t="inlineStr"/>
+          <t>NauseatingChurnNew_A</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Nauseating Churn</t>
+        </is>
+      </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Deal 9 damage to the Left and Right enemies. If wrong pigment was used, instead deal 12 damage.</t>
+          <t>Lowers the Opposing party member's max health by 2. Slightly heals the Opposing party members.</t>
         </is>
       </c>
     </row>
     <row r="135">
-      <c r="A135" t="inlineStr">
-        <is>
-          <t>Cleave the Bones</t>
-        </is>
-      </c>
+      <c r="A135" t="inlineStr"/>
       <c r="B135" t="inlineStr"/>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Deal 11 damage to the Left and Right enemies. If wrong pigment was used, instead deal 15 damage.</t>
+          <t>Upon death this enemy spawns 4 Neoplasms.</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Reap What You Set</t>
-        </is>
-      </c>
-      <c r="B136" t="inlineStr"/>
+          <t>DeafeningSilence_A</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Deafening Silence</t>
+        </is>
+      </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Deal 8 damage to the Left and Right enemies. If this party member is below half health, heal them 1 health.</t>
+          <t>Inflicts 1 Constricted to two random Opposing tiles and increase all the Opposing party member's health by 1. 
+Swaps this enemy's health color.</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Reap What You Laid</t>
-        </is>
-      </c>
-      <c r="B137" t="inlineStr"/>
+          <t>SloshAndGoop_A</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Slosh and Goop</t>
+        </is>
+      </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Deal 10 damage to the Left and Right enemies. If this party member is below half health, heal them 1 health.</t>
+          <t>If this enemy's health color is Red, deals a Painful amount of damage to all Right Opposing party members. If this enemy's health color is Yellow, deals a Painful amount of damage to all Left Opposing party members.</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Reap What You Sow</t>
-        </is>
-      </c>
-      <c r="B138" t="inlineStr"/>
+          <t>Thwart_A</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Thwart</t>
+        </is>
+      </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Deal 12 damage to the Left and Right enemies. If this party member is below half health, heal them 1 health.</t>
+          <t>This enemy attempts to grasp the Opposing party member between its fingers and applies an amount of Mutualism to itself equal to the party member's current health.</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Reap What You Did</t>
-        </is>
-      </c>
-      <c r="B139" t="inlineStr"/>
+          <t>Lob_A</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Lob</t>
+        </is>
+      </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Deal 14 damage to the Left and Right enemies. If this party member is below half health, heal them 1 health.</t>
+          <t>Deal an Agonizing amount of damage to the Opposing party member.
+Release the currently grasped party member.</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Outlast The Mark</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr"/>
+          <t>SlapofGod_A</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Slap of God</t>
+        </is>
+      </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Heal this party member 3 health, then reduce their maximum health by 1. Reduce Fatigue by 1.</t>
+          <t>\!*deep Inhale*\!
+Deals almost no damage to the Opposing party member. Inflict 1 Stun to the Opposing party member.</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Outlast The Target</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr"/>
+          <t>Recollection_A</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Recollection</t>
+        </is>
+      </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Heal this party member 5 health, then reduce their maximum health by 2. Reduce Fatigue by 2.</t>
+          <t>Inflict Stun to every party member with the Focus passive.
+Apply Focused to this enemy.</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Outlast The Quarry</t>
-        </is>
-      </c>
-      <c r="B142" t="inlineStr"/>
+          <t>Legion_A</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Legion</t>
+        </is>
+      </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Heal this party member 7 health, then reduce their maximum health by 3. Reduce Fatigue by 3.</t>
+          <t>Apply 1-2 Fire to the Opposing positions.
+Move Left or Right.
+Produce 1-2 Red pigment.
+\!For we are many\!</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Outlast The Victim</t>
-        </is>
-      </c>
-      <c r="B143" t="inlineStr"/>
+          <t>WalktheEarth_A</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Walk the Earth</t>
+        </is>
+      </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Heal this party member 9 health, then reduce their maximum health by 4. Reduce Fatigue by 4.</t>
+          <t>Move the Left and Right party members not Opposing this enemy closer to this enemy.
+Apply 1 Constricted to the Opposing positions.
+Produce 1-2 Red pigment.</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Unstitch Their Tendons</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr"/>
+          <t>CarbonTears_A</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Carbon Tears</t>
+        </is>
+      </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Deal 6 damage to the Opposing enemy. If this party member is below half health, inflict 1 Scar to them and refresh their abilities.</t>
+          <t>Apply 1 Fire to All party members that are Oil-Slicked.
+Inflict 1-2 Oil-Slicked to All party members not standing in Fire.
+Produce 1-2 Red pigment.</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Unstitch Their Sinew</t>
-        </is>
-      </c>
-      <c r="B145" t="inlineStr"/>
+          <t>Blood_A</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Blood</t>
+        </is>
+      </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Deal 8 damage to the Opposing enemy. If this party member is below half health, inflict 1 Scar to them and refresh their abilities.</t>
+          <t>Deals a Little amount of damage to the Opposing party member and Inflict 1 Fire to the Opposing position.
+If this enemy's health color is Red, instead Inflict 99 fire to the Opposing position and deal a Painful amount of damage to the Opposing party member.</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Unstitch Their Marrow</t>
-        </is>
-      </c>
-      <c r="B146" t="inlineStr"/>
+          <t>Bile_A</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Bile</t>
+        </is>
+      </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Deal 10 damage to the Opposing enemy. If this party member is below half health, inflict 1 Scar to them and refresh their abilities.</t>
+          <t>Inflict 1 Oil-slicked to the Opposing party member, and deal a Little amount of damage to the Opposing party member.
+If this enemy's health color is Yellow, instead deal a Painful amount of damage then Inflict 99 Oil-slicked to the Opposing party member.</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Unstitch Their Flesh</t>
-        </is>
-      </c>
-      <c r="B147" t="inlineStr"/>
+          <t>Arsenic_A</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Arsenic</t>
+        </is>
+      </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Deal 12 damage to the Opposing enemy. If this party member is below half health, inflict 1 Scar to them and refresh their abilities.</t>
+          <t>Inflict Curse to the Opposing party member.
+If this enemy's health color is Purple, reduce the Opposing party member's health to 20% of their max health and inflict them with Curse, and then deal Almost no damage to them.</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Brittle Leash</t>
-        </is>
-      </c>
-      <c r="B148" t="inlineStr"/>
+          <t>Salt_A</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Inflict the Opposing enemy with 1 Constricted and deal 5 damage to them.</t>
+          <t>Inflict 1 Ruptured to the Opposing party member, and move the Opposing party member Left or Right.
+If this enemy's health color is Blue, instead Apply 99 Ruptured to the Opposing party member, move this enemy Left or Right 3 times, and Deal a Painful amount of damage to the Opposing party member.\r</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Weak Leash</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr"/>
+          <t>FourHumors_A</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Four Humors</t>
+        </is>
+      </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Inflict the Opposing enemy with 2 Constricted and deal 7 damage to them.</t>
+          <t>Produce 3 Pigment of this enemy's health color.
+Move this enemy to the Left or Right.</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Strong Leash</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr"/>
+          <t>BroodParasite_A</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Brood Parasite</t>
+        </is>
+      </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Inflict the Opposing enemy with 2 Constricted and deal 9 damage to them.</t>
+          <t>Applies Parental to the Left or Right enemy.
+\!Sadist in the making.\!</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Unbreakable Leash</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr"/>
+          <t>ChildrenareCruel_A</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Children are Cruel</t>
+        </is>
+      </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Inflict the Opposing enemy with 2 Constricted and deal 11 damage to them.</t>
+          <t>If the Opposing party member has less than 14 health, reduces the Opposing party member to only 1 health.
+If their health is greater than 24, completely randomizes their health.</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Limply Whip</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr"/>
+          <t>ElaboratePrank_A</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Elaborate Prank</t>
+        </is>
+      </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>50% chance to deal 9 damage to the Opposing enemy. If successful, move the Opposing enemy to the Left or Right. Afterwards, 50% chance to deal 9 damage to the Opposing enemy.</t>
+          <t>Inflicts 1 of most Status and Field effects to the Opposing party member.</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Sluggishly Whip</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr"/>
+          <t>WarisDeception_A</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>War is Deception</t>
+        </is>
+      </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>60% chance to deal 11 damage to the Opposing enemy. If successful, move the Opposing enemy to the Left or Right. Afterwards, 60% chance to deal 11 damage to the Opposing enemy.</t>
+          <t>Perform a random ability from one of the other enemies in combat.</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Menacingly Whip</t>
-        </is>
-      </c>
-      <c r="B154" t="inlineStr"/>
+          <t>FromtheGarden_A</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>From the Garden</t>
+        </is>
+      </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>70% chance to deal 14 damage to the Opposing enemy. If successful, move the Opposing enemy to the Left or Right. Afterwards, 70% chance to deal 14 damage to the Opposing enemy.</t>
+          <t>Fully Heal all other enemies, deal damage to this enemy equal to amount healed.</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Terrifyingly Whip</t>
-        </is>
-      </c>
-      <c r="B155" t="inlineStr"/>
+          <t>WithintheGrid_A</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Within the Grid</t>
+        </is>
+      </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>75% chance to deal 16 damage to the Opposing enemy. If successful, move the Opposing enemy to the Left or Right. Afterwards, 75% chance to deal 16 damage to the Opposing enemy.</t>
+          <t>If this enemy's health color is Grey, change the health color of all other enemies to Grey and change this enemy's health color to Red.
+If this enemy's health color isn't Grey, change the health color of all other enemies to this enemy's health color and change this enemy's health color to Grey.</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Bloat Minutely</t>
-        </is>
-      </c>
-      <c r="B156" t="inlineStr"/>
+          <t>CradleofAffliction_A</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Cradle of Affliction</t>
+        </is>
+      </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>At the start of the next turn, deal 8, 12, or 16 damage to the Opposing enemy.</t>
+          <t>Applies 1 Divine protection to either this enemy or 2 Divine protection to all other enemies.</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Bloat Moderately</t>
-        </is>
-      </c>
-      <c r="B157" t="inlineStr"/>
+          <t>FirstSteps_A</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>First Steps</t>
+        </is>
+      </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>At the start of the next turn, deal 8, 12, or 16 damage to the Opposing and Left enemies.</t>
+          <t>Moves to the Left or Right. Increases the damage of \!Thump\! by 2.</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Bloat Majorly</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr"/>
+          <t>Thump_A</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Thump</t>
+        </is>
+      </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>At the start of the next turn, deal 8, 12, or 16 damage to the Opposing, Left, and Right enemies.</t>
+          <t>Deals a Painful amount of damage to the Opposing party member. Damage cascades to the Left and Right.</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Bloat Massively</t>
-        </is>
-      </c>
-      <c r="B159" t="inlineStr"/>
+          <t>CryPierceTheSky_A</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Cry, Pierce the Sky</t>
+        </is>
+      </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>At the start of the next turn, deal 8, 12, or 16 damage to the Opposing, Left, Far Left, Right, and Far Right enemies.</t>
+          <t>Forces all Revolas to stand. 
+If there are no Revolas present, produces 1 Blue Pigment and increases the damage of \!Thump\! by 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>ToreaMuscle_A</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Tore a Muscle</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>\!Strained too hard, tore a muscle clean...\!
+Deals a Little amount of damage to this enemy and inflicts 2 Scars to this enemy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>TrumpetsoftheApocalypse_A</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Trumpets of the Apocalypse</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Applies 2 Ruptured to all Opposing party members. Applies 0-3 Scars to all party members.
+\!Look at me. Look at me damn you.\!</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>BellowingWail_A</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Bellowing Wail</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Deals an Agonizing amount of damage to the Opposing party members.
+Applies 3 Scars to all Opposing party members and this enemy. 
+Applies 2-10 Shield randomly to each enemy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>InternalFluids_A</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Internal Fluids</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Inflicts 2 Oil-Slicked to all party members and 4 Ruptured to all Opposing party members.
+Applies 2 Scars to this enemy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>LastStand_A</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Last Stand</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>This enemy reveals the true extent to its injuries.
+\!I'll see you in Hell.\!</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Barter_A</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Barter</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Move this enemy to the Left.
+Deal a Little Indirect damage to the Opposing party member.
+If the Opposing party member has an item, permanetly change it to a random treasure item.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Trade_A</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Trade</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Move this enemy to the Right.
+Deal a Little Indirect damage to the Opposing party member.
+If the Opposing party member has an item, permanetly change it to a random treasure item.</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>FairPrice_A</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Fair Price</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Move this enemy Left or Right.
+Steal 3 coins from the Opposing party member. If the Opposing party member has an item, produce 6 coins.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>SockLeft_A</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Sock Left</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Deal a Painful amount of damage to the Left party member.</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>WallopRight_A</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Wallop Right</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Deal a Painful amount of damage to the Right party member.</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>WhiteNoise_A</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>White Noise</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>25% chance to Inflict 2 Constriced to each party member and enemy tile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>BabyMonitor_A</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Baby Monitor</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Deal a Painful amount of damage to the enemy(s) with the lowest health.</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>NewOrders_A</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>New Orders</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Deal a Painful amount of damage to the enemy(s) with the highest health.</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Caretaker_A</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Caretaker</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Heals all enemies with less health than this enemy. If this enemy has the lowest health, applies 10 Shield to it's position instead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>DrivethemDown_A</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Drive them Down</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Force the opposing party member into a tile with fire on it.
+Apply 1 Constricted and 1 Fire to that party member's tile.
+Produce 1 Red pigment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Pyromancy_A</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Pyromancy</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Moves all party members away from this enemy.
+Applies 0-2 fire to the opposing tile 3 times.
+Produce 1 Red pigment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>DeepBeat_A</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Deep Beat</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Apply 2 Frail to the Left and Right Opposing party members, and move them Left or Right.
+Deal a Painful amount of damage to the Middle opposing party member.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Seethe_A</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Seethe</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Apply 4 Ruptured to the Middle opposing party member, and move them Left or Right.</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>BellowingBallad_A</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Bellowing Ballad</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Move all party members to the Middle opposing slot.
+Apply 2 Frail to the Middle opposing party member, and 2 Ruptured to the Left and Right opposing party members.</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>BecometheRhythm_A</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Become the Rhythm</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Transforms into a performance of the Ungod.</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>CoinGun_A_0</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Coin Gun</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Consumes 1 coin, if successful. Deals 3 damage to the opposing enemy, and Refreshes this party member's abilities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>PostMotermGuardian_A</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Post-mortem Guardian</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Retribution for violence against infants(?).
+Moves this enemy to the Left or Right.
+Deals a Painful amount of damage to Opposing party members.
+Heals all infantile enemies 1 health.</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>BoneCrush_A</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Bone Crush</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Deals a Painful amount of damage to all Opposing party members. Inflict 2 Frail to all Opposing party members.</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>SoulDevour_A</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Soul Devour</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Consumes all pigment.
+Deal Indirect damage equal to how much pigment was consumed to the Opposing party members, the damage will be spread equally among them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Shudder_A</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Shudder</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Deals a Painful amount of damage to this enemy and ejects a Flarbleft.</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>BasalTear_A</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Basal Tear</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>\!My guts lay splattered across the floor, and it feels like how they're meant to be arranged by nature.\!
+Inflicts 2 Ruptured and deals a Painful amount of indirect damage to the Opposing party member.
+Moves this enemy to the Left or Right.</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>OthersideScreech_A</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Otherside Screech</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>\!I'm not my brain, I'm my eyes.\!
+Inflicts 3 Ruptured to the Left and Right party members.</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>DemonCircuit_A</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Demon Circuit</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>\!Coding for reflexes of long-obsolete terrors claw and shred their way out of my cells.\!
+Increases the duration of all negative status effects to the Left, Right, and Opposing party members by 1. 60% chance to Curse the Opposing party member.</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>TranshumanSubhuman_A</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>IsClose</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>The horrible mistake reveals itself.</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Inlapse_A</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Inlapse</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>The abomination hides into its ruined body.</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Decapitate_A</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Decapitate</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Deals a Little amount of Damage to the Opposing party member.
+Removes all Ruptured from the Opposing party member, heals them for the amount removed, and applies 2 Scars to them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Quarter_A</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Quarter</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Deals a Painful amount of Damage to the Right party member.
+If they are Ruptured, deals an Agonizing amount of Damage to them instead. 
+Moves this enemy to the Left.</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Dice_A</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Dice</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Deals a Painful amount of Damage to the Left party member.
+If the target party member is Ruptured, deal an Agonizing amount of Damage to them instead. 
+Moves this enemy to the Right.</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Whimsy_A</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Whimsy</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Remove all Shield from this enemy position.
+Apply 9 shield to this enemy's position.</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Shoo_A</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Shoo</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Move this enemy to the Left or Right.
+Deal a Painful amount of damage to the Opposing party member.
+Attempt to move back to the previous position.</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>WretchedTraitor_A</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Wretched Traitor</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Deal a Mortal amount of Shield-piercing damage to the Left and Right enemies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>WretchedTraitorAlt_A</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Wretched Traitor</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Deal a Mortal amount of Shield-piercing damage to the Left and Right enemies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>MarrowProber_A</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Marrow Prober</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Move this enemy to the Left or Right. Deal an Agonizing amount of Shield-piercing damage to the Left and Right enemies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>MarrowProberAlt_A</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Marrow Prober</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Move this enemy to the Left or Right. Deal an Agonizing amount of Shield-piercing damage to the Left and Right enemies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Iteatsaway_A</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>It eats away</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Decrease the Opposing party member's maximum health by 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>NoEscape_A</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>No Escape</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Deal a Little amount of damage to the Opposing party member.
+Inflict 2 Constricted to the opposing position.</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>CertainFate_A</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Certain Fate</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Curse the Opposing party member.</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Migraine_A</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Migraine</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Attempts to swap positions with a random Singing Stone. 
+Deals a Painful amount of damage to the Opposing party member.</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Cluster_A</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Cluster</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Deals a Painful amount of damage to this enemy and spawns 1-2 Singing Stones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Thunderclap_A</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Thunderclap</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Applies 3 Frail to all party members Opposing a Singing Stone.
+Spawns a Singing Stone if there are none</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Realize_A</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Realize</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Deals a Painful amount damage to the Left and Opposing party members.
+Moves this enemy to the Left.
+Bleeds 2 Red Pigment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Harrow_A</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Harrow</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Deals a Painful amount damage to the Right and Opposing party members.
+Moves this enemy to the Right.
+Bleeds 2 Red Pigment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>MetabolicHellfire_A</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Metabolic Hellfire</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Inflicts 4 Fire to the Central Opposing party member.
+Inflicts 1 Scar to the Central Opposing party member.</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>IntestinalSinge_A</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Intestinal Singe</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Inflicts 2 Fire to the Left and Right Opposing party members.</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>OrganShutDown_A</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Organ Shut-Down</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>\!Actually reduces heat\!
+Removes all Fire from this enemy's position and Greatly heals this enemy.
+Inflicts 1 Scar to all party members and 1 Fire to all empty party member slots.</t>
         </is>
       </c>
     </row>

</xml_diff>